<commit_message>
✨ xlsx: 数式の関数評価 (SUM / IF / ROUND / TEXT など 38 関数)
Formula に関数呼び出しと範囲引数を追加。SUM PRODUCT AVERAGE COUNT COUNTA
COUNTBLANK MIN MAX ABS INT SQRT MOD POWER ROUND ROUNDUP ROUNDDOWN IF IFERROR
AND OR NOT TRUE FALSE LEN UPPER LOWER TRIM LEFT RIGHT MID CONCAT CONCATENATE
TEXT VALUE ISBLANK ISNUMBER ISTEXT ISERROR。
範囲の中の文字列・真偽・空は数値関数では無視、直接の引数は Excel と同じく
型強制。単独のセル参照は 1 セルの範囲として扱う (AVERAGE(空) は #DIV/0!)。
引数区切りは , と ; の両方、関数名は大文字小文字を問わない。
未対応の関数 (VLOOKUP など)、定義名、列全体の範囲は従来どおり空 + 数式表示。
テスト 5 件 (41 テスト)、sample.xlsx に関数の行、README。

Closes #34

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017AqpV42wRhuHFKJS7vC5HZ
</commit_message>
<xml_diff>
--- a/Tests/viwTests/Fixtures/sample.xlsx
+++ b/Tests/viwTests/Fixtures/sample.xlsx
@@ -908,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1092,6 +1092,29 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>func2</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(B2&gt;100,"many","few")</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>ROUND(C5/7,2)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>COUNTA(A2:A9)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>TEXT(D2,"#,##0")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✨ xlsx: 数式の関数評価 (SUM / IF / ROUND / TEXT など 38 関数) (#40)
Formula に関数呼び出しと範囲引数を追加。SUM PRODUCT AVERAGE COUNT COUNTA
COUNTBLANK MIN MAX ABS INT SQRT MOD POWER ROUND ROUNDUP ROUNDDOWN IF IFERROR
AND OR NOT TRUE FALSE LEN UPPER LOWER TRIM LEFT RIGHT MID CONCAT CONCATENATE
TEXT VALUE ISBLANK ISNUMBER ISTEXT ISERROR。
範囲の中の文字列・真偽・空は数値関数では無視、直接の引数は Excel と同じく
型強制。単独のセル参照は 1 セルの範囲として扱う (AVERAGE(空) は #DIV/0!)。
引数区切りは , と ; の両方、関数名は大文字小文字を問わない。
未対応の関数 (VLOOKUP など)、定義名、列全体の範囲は従来どおり空 + 数式表示。
テスト 5 件 (41 テスト)、sample.xlsx に関数の行、README。

Closes #34


Claude-Session: https://claude.ai/code/session_017AqpV42wRhuHFKJS7vC5HZ

Co-authored-by: td72 <12109493+td72@users.noreply.github.com>
Co-authored-by: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tests/viwTests/Fixtures/sample.xlsx
+++ b/Tests/viwTests/Fixtures/sample.xlsx
@@ -908,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1092,6 +1092,29 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>func2</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(B2&gt;100,"many","few")</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>ROUND(C5/7,2)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>COUNTA(A2:A9)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>TEXT(D2,"#,##0")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>